<commit_message>
add AsDataTrace extension and move profile-datatype folder 0232b85f0c5ba7464dd24d2c2b1443af98aea67b
</commit_message>
<xml_diff>
--- a/ig/nr-deploy-1.0.0-ballot/StructureDefinition-as-location.xlsx
+++ b/ig/nr-deploy-1.0.0-ballot/StructureDefinition-as-location.xlsx
@@ -9,11 +9,14 @@
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AL$49</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1402" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1707" uniqueCount="341">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-26T12:00:53+00:00</t>
+    <t>2023-06-02T12:29:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -301,20 +304,216 @@
 </t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Location.meta.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Location.meta.extension</t>
+  </si>
+  <si>
+    <t>extensions
+user content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension
+</t>
+  </si>
+  <si>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
+  </si>
+  <si>
+    <t>Location.meta.extension:as-data-trace</t>
+  </si>
+  <si>
+    <t>as-data-trace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-data-trace}
+</t>
+  </si>
+  <si>
+    <t>DataTrace</t>
+  </si>
+  <si>
+    <t>Informe sur l'origine de la donnée (Autorité d'Enregistrement (AE) et Système d'Information (SI))..</t>
+  </si>
+  <si>
+    <t>Location.meta.versionId</t>
+  </si>
+  <si>
+    <t>Version specific identifier</t>
+  </si>
+  <si>
+    <t>The version specific identifier, as it appears in the version portion of the URL. This value changes when the resource is created, updated, or deleted.</t>
+  </si>
+  <si>
+    <t>The server assigns this value, and ignores what the client specifies, except in the case that the server is imposing version integrity on updates/deletes.</t>
+  </si>
+  <si>
+    <t>Meta.versionId</t>
+  </si>
+  <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Location.implicitRules</t>
+    <t>Location.meta.lastUpdated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instant
+</t>
+  </si>
+  <si>
+    <t>When the resource version last changed</t>
+  </si>
+  <si>
+    <t>When the resource last changed - e.g. when the version changed.</t>
+  </si>
+  <si>
+    <t>This value is always populated except when the resource is first being created. The server / resource manager sets this value; what a client provides is irrelevant. This is equivalent to the HTTP Last-Modified and SHOULD have the same value on a [read](http://hl7.org/fhir/R4/http.html#read) interaction.</t>
+  </si>
+  <si>
+    <t>Meta.lastUpdated</t>
+  </si>
+  <si>
+    <t>Location.meta.source</t>
   </si>
   <si>
     <t xml:space="preserve">uri
 </t>
   </si>
   <si>
+    <t>Identifies where the resource comes from</t>
+  </si>
+  <si>
+    <t>A uri that identifies the source system of the resource. This provides a minimal amount of [Provenance](http://hl7.org/fhir/R4/provenance.html#) information that can be used to track or differentiate the source of information in the resource. The source may identify another FHIR server, document, message, database, etc.</t>
+  </si>
+  <si>
+    <t>In the provenance resource, this corresponds to Provenance.entity.what[x]. The exact use of the source (and the implied Provenance.entity.role) is left to implementer discretion. Only one nominated source is allowed; for additional provenance details, a full Provenance resource should be used. 
+This element can be used to indicate where the current master source of a resource that has a canonical URL if the resource is no longer hosted at the canonical URL.</t>
+  </si>
+  <si>
+    <t>Meta.source</t>
+  </si>
+  <si>
+    <t>Location.meta.profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canonical(StructureDefinition)
+</t>
+  </si>
+  <si>
+    <t>Profiles this resource claims to conform to</t>
+  </si>
+  <si>
+    <t>A list of profiles (references to [StructureDefinition](http://hl7.org/fhir/R4/structuredefinition.html#) resources) that this resource claims to conform to. The URL is a reference to [StructureDefinition.url](http://hl7.org/fhir/R4/structuredefinition-definitions.html#StructureDefinition.url).</t>
+  </si>
+  <si>
+    <t>It is up to the server and/or other infrastructure of policy to determine whether/how these claims are verified and/or updated over time.  The list of profile URLs is a set.</t>
+  </si>
+  <si>
+    <t>Meta.profile</t>
+  </si>
+  <si>
+    <t>Location.meta.security</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Security Labels applied to this resource</t>
+  </si>
+  <si>
+    <t>Security labels applied to this resource. These tags connect specific resources to the overall security policy and infrastructure.</t>
+  </si>
+  <si>
+    <t>The security labels can be updated without changing the stated version of the resource. The list of security labels is a set. Uniqueness is based the system/code, and version and display are ignored.</t>
+  </si>
+  <si>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>Security Labels from the Healthcare Privacy and Security Classification System.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/security-labels</t>
+  </si>
+  <si>
+    <t>Meta.security</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>Location.meta.tag</t>
+  </si>
+  <si>
+    <t>Tags applied to this resource</t>
+  </si>
+  <si>
+    <t>Tags applied to this resource. Tags are intended to be used to identify and relate resources to process and workflow, and applications are not required to consider the tags when interpreting the meaning of a resource.</t>
+  </si>
+  <si>
+    <t>The tags can be updated without changing the stated version of the resource. The list of tags is a set. Uniqueness is based the system/code, and version and display are ignored.</t>
+  </si>
+  <si>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Codes that represent various types of tags, commonly workflow-related; e.g. "Needs review by Dr. Jones".</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/common-tags</t>
+  </si>
+  <si>
+    <t>Meta.tag</t>
+  </si>
+  <si>
+    <t>Location.implicitRules</t>
+  </si>
+  <si>
     <t>A set of rules under which this content was created</t>
   </si>
   <si>
@@ -325,9 +524,6 @@
   </si>
   <si>
     <t>Resource.implicitRules</t>
-  </si>
-  <si>
-    <t>n/a</t>
   </si>
   <si>
     <t>Location.language</t>
@@ -410,38 +606,10 @@
     <t>Location.extension</t>
   </si>
   <si>
-    <t>extensions
-user content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension
-</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
     <t>May be used to represent additional information that is not part of the basic definition of the resource. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
   </si>
   <si>
-    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:url}
-</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
     <t>DomainResource.extension</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
     <t>Location.modifierExtension</t>
@@ -512,10 +680,6 @@
     <t>Location.operationalStatus</t>
   </si>
   <si>
-    <t xml:space="preserve">Coding
-</t>
-  </si>
-  <si>
     <t>The operational status of the location (typically only for a bed/room)</t>
   </si>
   <si>
@@ -531,14 +695,7 @@
     <t>http://terminology.hl7.org/ValueSet/v2-0116</t>
   </si>
   <si>
-    <t>CV</t>
-  </si>
-  <si>
     <t>Location.name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">string
-</t>
   </si>
   <si>
     <t>Name of the location as used by humans</t>
@@ -624,9 +781,6 @@
     <t>Not all terminology uses fit this general pattern. In some cases, models should not use CodeableConcept and use Coding directly and provide their own structure for managing text, codings, translations and the relationship between elements and pre- and post-coordination.</t>
   </si>
   <si>
-    <t>extensible</t>
-  </si>
-  <si>
     <t>http://terminology.hl7.org/ValueSet/v3-ServiceDeliveryLocationRoleType</t>
   </si>
   <si>
@@ -687,9 +841,6 @@
     <t>For purposes of showing relevant locations in queries, we need to categorize locations.</t>
   </si>
   <si>
-    <t>example</t>
-  </si>
-  <si>
     <t>Physical form of the location.</t>
   </si>
   <si>
@@ -721,22 +872,7 @@
     <t>Location.position.id</t>
   </si>
   <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
     <t>Location.position.extension</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>Location.position.modifierExtension</t>
@@ -1070,6 +1206,21 @@
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="22"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="22"/>
+        <i val="true"/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1235,12 +1386,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL40"/>
+  <dimension ref="A1:AL49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="42.98046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="42.98046875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="12.66015625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="13.30859375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="39.9140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>
@@ -1262,7 +1413,7 @@
     <col min="22" max="22" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="84.6796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="67.80078125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
@@ -1393,7 +1544,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="true">
       <c r="A2" t="s" s="2">
         <v>28</v>
       </c>
@@ -1499,7 +1650,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="true">
       <c r="A3" t="s" s="2">
         <v>80</v>
       </c>
@@ -1607,7 +1758,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
         <v>88</v>
       </c>
@@ -1704,21 +1855,21 @@
         <v>93</v>
       </c>
       <c r="AJ4" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AK4" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="AK4" t="s" s="2">
+      <c r="AL4" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" hidden="true">
+      <c r="A5" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="AL4" t="s" s="2">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="2">
-        <v>96</v>
-      </c>
       <c r="B5" t="s" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s" s="2">
@@ -1735,23 +1886,21 @@
         <v>73</v>
       </c>
       <c r="I5" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K5" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L5" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="L5" t="s" s="2">
+      <c r="M5" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="M5" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N5" t="s" s="2">
-        <v>100</v>
-      </c>
+      <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" t="s" s="2">
         <v>73</v>
@@ -1800,7 +1949,7 @@
         <v>73</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>74</v>
@@ -1809,35 +1958,35 @@
         <v>81</v>
       </c>
       <c r="AI5" t="s" s="2">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="AK5" t="s" s="2">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AL5" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>73</v>
@@ -1849,16 +1998,16 @@
         <v>73</v>
       </c>
       <c r="K6" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="L6" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="L6" t="s" s="2">
+      <c r="M6" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="M6" t="s" s="2">
+      <c r="N6" t="s" s="2">
         <v>106</v>
-      </c>
-      <c r="N6" t="s" s="2">
-        <v>107</v>
       </c>
       <c r="O6" s="2"/>
       <c r="P6" t="s" s="2">
@@ -1884,61 +2033,63 @@
         <v>73</v>
       </c>
       <c r="X6" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y6" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z6" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA6" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB6" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AC6" t="s" s="2">
         <v>108</v>
       </c>
-      <c r="Y6" t="s" s="2">
+      <c r="AD6" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE6" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="Z6" t="s" s="2">
+      <c r="AF6" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="AA6" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB6" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC6" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD6" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE6" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF6" t="s" s="2">
-        <v>111</v>
-      </c>
       <c r="AG6" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH6" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI6" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ6" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AK6" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="AK6" t="s" s="2">
-        <v>102</v>
-      </c>
       <c r="AL6" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
         <v>112</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>101</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>113</v>
+      </c>
       <c r="D7" t="s" s="2">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" t="s" s="2">
@@ -1948,7 +2099,7 @@
         <v>81</v>
       </c>
       <c r="H7" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="I7" t="s" s="2">
         <v>73</v>
@@ -1965,9 +2116,7 @@
       <c r="M7" t="s" s="2">
         <v>116</v>
       </c>
-      <c r="N7" t="s" s="2">
-        <v>117</v>
-      </c>
+      <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
         <v>73</v>
@@ -2016,44 +2165,44 @@
         <v>73</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH7" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI7" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="AK7" t="s" s="2">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="AL7" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
-        <v>121</v>
+        <v>73</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>73</v>
@@ -2062,19 +2211,19 @@
         <v>73</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -2124,44 +2273,44 @@
         <v>73</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI8" t="s" s="2">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AL8" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
-        <v>128</v>
+        <v>73</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>73</v>
@@ -2170,19 +2319,19 @@
         <v>73</v>
       </c>
       <c r="J9" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -2220,81 +2369,79 @@
         <v>73</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="AC9" t="s" s="2">
-        <v>134</v>
+        <v>73</v>
       </c>
       <c r="AD9" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AL9" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
-        <v>128</v>
+        <v>73</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J10" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="J10" t="s" s="2">
-        <v>73</v>
-      </c>
       <c r="K10" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="O10" t="s" s="2">
-        <v>141</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
         <v>73</v>
       </c>
@@ -2330,45 +2477,45 @@
         <v>73</v>
       </c>
       <c r="AB10" t="s" s="2">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="AC10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE10" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF10" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="AD10" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE10" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="AF10" t="s" s="2">
-        <v>142</v>
-      </c>
       <c r="AG10" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI10" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AL10" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2391,18 +2538,18 @@
         <v>82</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>146</v>
-      </c>
-      <c r="N11" s="2"/>
-      <c r="O11" t="s" s="2">
-        <v>147</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="N11" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
         <v>73</v>
       </c>
@@ -2450,7 +2597,7 @@
         <v>73</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>74</v>
@@ -2462,21 +2609,21 @@
         <v>93</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>148</v>
+        <v>100</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>149</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2487,28 +2634,28 @@
         <v>74</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I12" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -2534,13 +2681,13 @@
         <v>73</v>
       </c>
       <c r="X12" t="s" s="2">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="Y12" t="s" s="2">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="Z12" t="s" s="2">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>73</v>
@@ -2558,33 +2705,33 @@
         <v>73</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>158</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2595,7 +2742,7 @@
         <v>74</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>73</v>
@@ -2607,16 +2754,16 @@
         <v>82</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2642,13 +2789,13 @@
         <v>73</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>108</v>
+        <v>155</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>73</v>
@@ -2666,33 +2813,33 @@
         <v>73</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH13" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI13" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>158</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2709,22 +2856,22 @@
         <v>73</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J14" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>168</v>
+        <v>130</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
@@ -2774,7 +2921,7 @@
         <v>73</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>74</v>
@@ -2786,21 +2933,21 @@
         <v>93</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>172</v>
+        <v>100</v>
       </c>
       <c r="AL14" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2811,7 +2958,7 @@
         <v>74</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>73</v>
@@ -2823,20 +2970,18 @@
         <v>73</v>
       </c>
       <c r="K15" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="L15" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="M15" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="N15" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="L15" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="M15" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="O15" t="s" s="2">
-        <v>177</v>
-      </c>
+      <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>73</v>
       </c>
@@ -2860,13 +3005,13 @@
         <v>73</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>73</v>
+        <v>169</v>
       </c>
       <c r="Y15" t="s" s="2">
-        <v>73</v>
+        <v>170</v>
       </c>
       <c r="Z15" t="s" s="2">
-        <v>73</v>
+        <v>171</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>73</v>
@@ -2884,37 +3029,37 @@
         <v>73</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>172</v>
+        <v>100</v>
       </c>
       <c r="AL15" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>73</v>
+        <v>174</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
@@ -2930,23 +3075,21 @@
         <v>73</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="O16" t="s" s="2">
-        <v>181</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
         <v>73</v>
       </c>
@@ -2994,7 +3137,7 @@
         <v>73</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>74</v>
@@ -3006,32 +3149,32 @@
         <v>93</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AL16" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
-        <v>73</v>
+        <v>182</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H17" t="s" s="2">
         <v>73</v>
@@ -3040,10 +3183,10 @@
         <v>73</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>104</v>
+        <v>183</v>
       </c>
       <c r="L17" t="s" s="2">
         <v>184</v>
@@ -3054,9 +3197,7 @@
       <c r="N17" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="O17" t="s" s="2">
-        <v>187</v>
-      </c>
+      <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
         <v>73</v>
       </c>
@@ -3080,61 +3221,61 @@
         <v>73</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>154</v>
+        <v>73</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>185</v>
+        <v>73</v>
       </c>
       <c r="Z17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>187</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AK17" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AL17" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" hidden="true">
+      <c r="A18" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="AA17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="AG17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AH17" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI17" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ17" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK17" t="s" s="2">
-        <v>189</v>
-      </c>
-      <c r="AL17" t="s" s="2">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="2">
-        <v>191</v>
-      </c>
       <c r="B18" t="s" s="2">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3150,19 +3291,19 @@
         <v>73</v>
       </c>
       <c r="J18" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>192</v>
+        <v>103</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>195</v>
+        <v>106</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3188,31 +3329,31 @@
         <v>73</v>
       </c>
       <c r="X18" t="s" s="2">
-        <v>196</v>
+        <v>73</v>
       </c>
       <c r="Y18" t="s" s="2">
-        <v>194</v>
+        <v>73</v>
       </c>
       <c r="Z18" t="s" s="2">
-        <v>197</v>
+        <v>73</v>
       </c>
       <c r="AA18" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AB18" t="s" s="2">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AC18" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="AD18" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE18" t="s" s="2">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>74</v>
@@ -3224,25 +3365,25 @@
         <v>93</v>
       </c>
       <c r="AJ18" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AK18" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="AK18" t="s" s="2">
-        <v>198</v>
-      </c>
       <c r="AL18" t="s" s="2">
-        <v>190</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3255,22 +3396,26 @@
         <v>73</v>
       </c>
       <c r="I19" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J19" t="s" s="2">
         <v>73</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>200</v>
+        <v>103</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
+        <v>193</v>
+      </c>
+      <c r="N19" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="O19" t="s" s="2">
+        <v>194</v>
+      </c>
       <c r="P19" t="s" s="2">
         <v>73</v>
       </c>
@@ -3306,19 +3451,19 @@
         <v>73</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="AC19" t="s" s="2">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="AD19" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>74</v>
@@ -3330,21 +3475,21 @@
         <v>93</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>203</v>
+        <v>111</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>204</v>
+        <v>94</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3355,7 +3500,7 @@
         <v>74</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>73</v>
@@ -3364,22 +3509,20 @@
         <v>73</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>208</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>209</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="N20" s="2"/>
       <c r="O20" t="s" s="2">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>73</v>
@@ -3428,33 +3571,33 @@
         <v>73</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>73</v>
+        <v>202</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3471,26 +3614,24 @@
         <v>73</v>
       </c>
       <c r="I21" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="J21" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>192</v>
+        <v>165</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="O21" t="s" s="2">
-        <v>215</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>73</v>
       </c>
@@ -3514,13 +3655,13 @@
         <v>73</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>73</v>
@@ -3538,7 +3679,7 @@
         <v>73</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>74</v>
@@ -3550,21 +3691,21 @@
         <v>93</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3584,21 +3725,21 @@
         <v>73</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>221</v>
+        <v>142</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>223</v>
-      </c>
-      <c r="N22" s="2"/>
-      <c r="O22" t="s" s="2">
-        <v>224</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>73</v>
       </c>
@@ -3622,13 +3763,13 @@
         <v>73</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>73</v>
+        <v>169</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>73</v>
+        <v>216</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>73</v>
+        <v>217</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>73</v>
@@ -3646,7 +3787,7 @@
         <v>73</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>74</v>
@@ -3658,21 +3799,21 @@
         <v>93</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>73</v>
+        <v>211</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3692,18 +3833,20 @@
         <v>73</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>168</v>
+        <v>96</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="N23" s="2"/>
+        <v>220</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>221</v>
+      </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>73</v>
@@ -3752,7 +3895,7 @@
         <v>73</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>74</v>
@@ -3761,28 +3904,28 @@
         <v>81</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>102</v>
+        <v>222</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>128</v>
+        <v>73</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
@@ -3801,18 +3944,20 @@
         <v>73</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>130</v>
+        <v>224</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="O24" s="2"/>
+        <v>226</v>
+      </c>
+      <c r="O24" t="s" s="2">
+        <v>227</v>
+      </c>
       <c r="P24" t="s" s="2">
         <v>73</v>
       </c>
@@ -3848,19 +3993,19 @@
         <v>73</v>
       </c>
       <c r="AB24" t="s" s="2">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="AC24" t="s" s="2">
-        <v>134</v>
+        <v>73</v>
       </c>
       <c r="AD24" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE24" t="s" s="2">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>74</v>
@@ -3872,56 +4017,56 @@
         <v>93</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>95</v>
+        <v>222</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>234</v>
+        <v>73</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>73</v>
       </c>
       <c r="I25" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="J25" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>132</v>
+        <v>206</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>141</v>
+        <v>231</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>73</v>
@@ -3970,33 +4115,33 @@
         <v>73</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>95</v>
+        <v>232</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4004,7 +4149,7 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>81</v>
@@ -4016,21 +4161,23 @@
         <v>73</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>239</v>
+        <v>165</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="O26" s="2"/>
+        <v>236</v>
+      </c>
+      <c r="O26" t="s" s="2">
+        <v>237</v>
+      </c>
       <c r="P26" t="s" s="2">
         <v>73</v>
       </c>
@@ -4054,13 +4201,13 @@
         <v>73</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>73</v>
+        <v>207</v>
       </c>
       <c r="Y26" t="s" s="2">
-        <v>73</v>
+        <v>235</v>
       </c>
       <c r="Z26" t="s" s="2">
-        <v>73</v>
+        <v>238</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>73</v>
@@ -4078,10 +4225,10 @@
         <v>73</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>81</v>
@@ -4090,21 +4237,21 @@
         <v>93</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>73</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4112,10 +4259,10 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>73</v>
@@ -4124,19 +4271,19 @@
         <v>73</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="M27" t="s" s="2">
+        <v>244</v>
+      </c>
+      <c r="N27" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>246</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -4162,13 +4309,13 @@
         <v>73</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>73</v>
+        <v>146</v>
       </c>
       <c r="Y27" t="s" s="2">
-        <v>73</v>
+        <v>244</v>
       </c>
       <c r="Z27" t="s" s="2">
-        <v>73</v>
+        <v>246</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>73</v>
@@ -4186,33 +4333,33 @@
         <v>73</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="AG27" t="s" s="2">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>73</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4223,7 +4370,7 @@
         <v>74</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>73</v>
@@ -4235,17 +4382,15 @@
         <v>73</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>242</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>73</v>
@@ -4294,33 +4439,33 @@
         <v>73</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>94</v>
+        <v>252</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4340,22 +4485,22 @@
         <v>73</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>73</v>
@@ -4404,7 +4549,7 @@
         <v>73</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>74</v>
@@ -4416,21 +4561,21 @@
         <v>93</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>256</v>
+        <v>122</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4450,22 +4595,22 @@
         <v>73</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>73</v>
@@ -4490,13 +4635,13 @@
         <v>73</v>
       </c>
       <c r="X30" t="s" s="2">
-        <v>73</v>
+        <v>155</v>
       </c>
       <c r="Y30" t="s" s="2">
-        <v>73</v>
+        <v>265</v>
       </c>
       <c r="Z30" t="s" s="2">
-        <v>73</v>
+        <v>266</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>73</v>
@@ -4514,7 +4659,7 @@
         <v>73</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>74</v>
@@ -4526,21 +4671,21 @@
         <v>93</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>256</v>
+        <v>122</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>73</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4551,7 +4696,7 @@
         <v>74</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H31" t="s" s="2">
         <v>73</v>
@@ -4563,18 +4708,18 @@
         <v>73</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>221</v>
+        <v>269</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="O31" s="2"/>
+        <v>271</v>
+      </c>
+      <c r="N31" s="2"/>
+      <c r="O31" t="s" s="2">
+        <v>272</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>73</v>
       </c>
@@ -4622,33 +4767,33 @@
         <v>73</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI31" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4671,13 +4816,13 @@
         <v>73</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>168</v>
+        <v>96</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>227</v>
+        <v>97</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>228</v>
+        <v>98</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4728,7 +4873,7 @@
         <v>73</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>229</v>
+        <v>99</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>74</v>
@@ -4743,22 +4888,22 @@
         <v>73</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -4777,16 +4922,16 @@
         <v>73</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>231</v>
+        <v>105</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4824,19 +4969,19 @@
         <v>73</v>
       </c>
       <c r="AB33" t="s" s="2">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="AC33" t="s" s="2">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="AD33" t="s" s="2">
         <v>73</v>
       </c>
       <c r="AE33" t="s" s="2">
-        <v>135</v>
+        <v>109</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>232</v>
+        <v>110</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>74</v>
@@ -4848,25 +4993,25 @@
         <v>93</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>234</v>
+        <v>277</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -4885,19 +5030,19 @@
         <v>82</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>235</v>
+        <v>278</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>236</v>
+        <v>279</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>141</v>
+        <v>194</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>73</v>
@@ -4946,7 +5091,7 @@
         <v>73</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>237</v>
+        <v>280</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>74</v>
@@ -4958,21 +5103,21 @@
         <v>93</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4980,10 +5125,10 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>73</v>
@@ -4995,16 +5140,16 @@
         <v>73</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>104</v>
+        <v>282</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>153</v>
+        <v>285</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5030,13 +5175,13 @@
         <v>73</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>154</v>
+        <v>73</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>276</v>
+        <v>73</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>277</v>
+        <v>73</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>73</v>
@@ -5054,33 +5199,33 @@
         <v>73</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5088,7 +5233,7 @@
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G36" t="s" s="2">
         <v>81</v>
@@ -5103,15 +5248,17 @@
         <v>73</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>281</v>
-      </c>
-      <c r="N36" s="2"/>
+        <v>289</v>
+      </c>
+      <c r="N36" t="s" s="2">
+        <v>285</v>
+      </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>73</v>
@@ -5160,10 +5307,10 @@
         <v>73</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="AG36" t="s" s="2">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="AH36" t="s" s="2">
         <v>81</v>
@@ -5172,21 +5319,21 @@
         <v>93</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5209,15 +5356,17 @@
         <v>73</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="M37" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="N37" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>73</v>
@@ -5266,7 +5415,7 @@
         <v>73</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>74</v>
@@ -5278,21 +5427,21 @@
         <v>93</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5312,19 +5461,23 @@
         <v>73</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
+        <v>296</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="O38" t="s" s="2">
+        <v>298</v>
+      </c>
       <c r="P38" t="s" s="2">
         <v>73</v>
       </c>
@@ -5372,7 +5525,7 @@
         <v>73</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>74</v>
@@ -5384,21 +5537,21 @@
         <v>93</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>94</v>
+        <v>299</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>269</v>
+        <v>300</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5421,18 +5574,20 @@
         <v>73</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>168</v>
+        <v>302</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="O39" s="2"/>
+        <v>305</v>
+      </c>
+      <c r="O39" t="s" s="2">
+        <v>306</v>
+      </c>
       <c r="P39" t="s" s="2">
         <v>73</v>
       </c>
@@ -5480,7 +5635,7 @@
         <v>73</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>74</v>
@@ -5492,21 +5647,21 @@
         <v>93</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>94</v>
+        <v>299</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>102</v>
+        <v>307</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5529,20 +5684,18 @@
         <v>73</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>293</v>
+        <v>269</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>296</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>73</v>
       </c>
@@ -5590,7 +5743,7 @@
         <v>73</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>74</v>
@@ -5602,16 +5755,1002 @@
         <v>93</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>256</v>
+        <v>122</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="AL40" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" hidden="true">
+      <c r="A41" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K41" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
+      <c r="P41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF41" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="42" hidden="true">
+      <c r="A42" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K42" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="O42" s="2"/>
+      <c r="P42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB42" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AC42" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AD42" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE42" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AF42" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="AG42" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH42" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI42" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ42" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="43" hidden="true">
+      <c r="A43" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" t="s" s="2">
+        <v>277</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I43" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="J43" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="K43" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="O43" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="P43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q43" s="2"/>
+      <c r="R43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF43" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>317</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="O44" s="2"/>
+      <c r="P44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="46" hidden="true">
+      <c r="A46" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="47" hidden="true">
+      <c r="A47" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
+      <c r="P47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>312</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" hidden="true">
+      <c r="A48" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K48" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="O48" s="2"/>
+      <c r="P48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q48" s="2"/>
+      <c r="R48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF48" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK48" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="49" hidden="true">
+      <c r="A49" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="O49" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="P49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="AL49" t="s" s="2">
         <v>73</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AL49">
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="26">
+      <filters blank="true"/>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:AI48">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$G2&lt;&gt;"Y"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$Q2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>